<commit_message>
Minor fixes to first draft
Minor fixes to first draft rev 1.0
Create versions with .15CE extension (identical to .mem)
</commit_message>
<xml_diff>
--- a/engineering_basics/dsp_windows/dsp_windows_smaller.xlsx
+++ b/engineering_basics/dsp_windows/dsp_windows_smaller.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="DSP Windows" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="DSP Windows (smaller)" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Sanity" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -1448,16 +1448,16 @@
     <t xml:space="preserve">E[2]</t>
   </si>
   <si>
+    <t xml:space="preserve">bins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Processing Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E[3]</t>
+  </si>
+  <si>
     <t xml:space="preserve">power</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Processing Loss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E[3]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dB</t>
   </si>
   <si>
     <t xml:space="preserve">Scalloping Loss</t>
@@ -1491,16 +1491,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="000"/>
     <numFmt numFmtId="166" formatCode="@"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1615,12 +1617,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF333333"/>
@@ -1675,6 +1671,7 @@
       <sz val="11"/>
       <name val="Consolas"/>
       <family val="3"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2136,35 +2133,39 @@
     <xf numFmtId="164" fontId="16" fillId="7" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="7" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="7" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="15" borderId="8" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="15" borderId="8" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="9" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="9" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2172,99 +2173,95 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="18" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="23" fillId="18" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="18" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="18" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="14" xfId="61" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="19" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="19" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="18" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="18" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="18" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="7" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="18" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="7" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="18" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="14" xfId="61" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="19" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="19" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="18" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="18" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="7" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="18" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="7" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2272,11 +2269,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2608,7 +2609,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="n">
         <v>1</v>
       </c>
@@ -2634,7 +2635,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="n">
         <v>2</v>
       </c>
@@ -2660,7 +2661,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="n">
         <v>3</v>
       </c>
@@ -2686,7 +2687,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="n">
         <v>4</v>
       </c>
@@ -2712,7 +2713,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="n">
         <v>5</v>
       </c>
@@ -2738,7 +2739,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="n">
         <v>6</v>
       </c>
@@ -2764,7 +2765,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="n">
         <v>7</v>
       </c>
@@ -2790,7 +2791,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="n">
         <v>8</v>
       </c>
@@ -2816,7 +2817,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="n">
         <v>9</v>
       </c>
@@ -2842,7 +2843,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="n">
         <v>10</v>
       </c>
@@ -2868,7 +2869,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="n">
         <v>11</v>
       </c>
@@ -2894,7 +2895,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="n">
         <v>12</v>
       </c>
@@ -2914,7 +2915,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="n">
         <v>13</v>
       </c>
@@ -2940,7 +2941,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="n">
         <v>14</v>
       </c>
@@ -2966,7 +2967,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="n">
         <v>15</v>
       </c>
@@ -2992,7 +2993,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="n">
         <v>16</v>
       </c>
@@ -3018,7 +3019,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="n">
         <v>17</v>
       </c>
@@ -3044,7 +3045,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="n">
         <v>18</v>
       </c>
@@ -3070,7 +3071,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="n">
         <v>19</v>
       </c>
@@ -3096,7 +3097,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="n">
         <v>20</v>
       </c>
@@ -3122,7 +3123,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="n">
         <v>21</v>
       </c>
@@ -3148,7 +3149,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="n">
         <v>22</v>
       </c>
@@ -3174,7 +3175,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="n">
         <v>23</v>
       </c>
@@ -3200,7 +3201,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="n">
         <v>24</v>
       </c>
@@ -3226,7 +3227,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="n">
         <v>25</v>
       </c>
@@ -3252,7 +3253,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="n">
         <v>26</v>
       </c>
@@ -3278,7 +3279,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="n">
         <v>27</v>
       </c>
@@ -3304,7 +3305,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="n">
         <v>28</v>
       </c>
@@ -3330,7 +3331,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="n">
         <v>29</v>
       </c>
@@ -3356,7 +3357,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="n">
         <v>30</v>
       </c>
@@ -3382,7 +3383,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="n">
         <v>31</v>
       </c>
@@ -3408,7 +3409,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="n">
         <v>32</v>
       </c>
@@ -3434,7 +3435,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="n">
         <v>33</v>
       </c>
@@ -3460,7 +3461,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="n">
         <v>34</v>
       </c>
@@ -3486,7 +3487,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="n">
         <v>35</v>
       </c>
@@ -3512,7 +3513,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="n">
         <v>36</v>
       </c>
@@ -3538,7 +3539,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="n">
         <v>37</v>
       </c>
@@ -3564,7 +3565,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="n">
         <v>38</v>
       </c>
@@ -3590,7 +3591,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="n">
         <v>39</v>
       </c>
@@ -3616,7 +3617,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="8" t="n">
         <v>40</v>
       </c>
@@ -3634,7 +3635,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="n">
         <v>41</v>
       </c>
@@ -3660,7 +3661,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="n">
         <v>42</v>
       </c>
@@ -3686,7 +3687,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="n">
         <v>43</v>
       </c>
@@ -3712,7 +3713,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="n">
         <v>44</v>
       </c>
@@ -3738,7 +3739,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="n">
         <v>45</v>
       </c>
@@ -3764,7 +3765,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="n">
         <v>46</v>
       </c>
@@ -3790,7 +3791,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="n">
         <v>47</v>
       </c>
@@ -3816,7 +3817,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="n">
         <v>48</v>
       </c>
@@ -3842,7 +3843,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="n">
         <v>49</v>
       </c>
@@ -3868,7 +3869,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="8" t="n">
         <v>50</v>
       </c>
@@ -3894,7 +3895,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="n">
         <v>51</v>
       </c>
@@ -3920,7 +3921,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="n">
         <v>52</v>
       </c>
@@ -3946,7 +3947,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="n">
         <v>53</v>
       </c>
@@ -3972,7 +3973,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="n">
         <v>54</v>
       </c>
@@ -3998,7 +3999,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="n">
         <v>55</v>
       </c>
@@ -4024,7 +4025,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="8" t="n">
         <v>56</v>
       </c>
@@ -4048,7 +4049,7 @@
       </c>
       <c r="H57" s="17"/>
     </row>
-    <row r="58" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="8" t="n">
         <v>57</v>
       </c>
@@ -4071,7 +4072,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="n">
         <v>58</v>
       </c>
@@ -4094,7 +4095,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="n">
         <v>59</v>
       </c>
@@ -4120,7 +4121,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="n">
         <v>60</v>
       </c>
@@ -4144,7 +4145,7 @@
       </c>
       <c r="H61" s="17"/>
     </row>
-    <row r="62" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="n">
         <v>61</v>
       </c>
@@ -4167,7 +4168,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="n">
         <v>62</v>
       </c>
@@ -4190,7 +4191,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="n">
         <v>63</v>
       </c>
@@ -4213,7 +4214,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="8" t="n">
         <v>64</v>
       </c>
@@ -4236,7 +4237,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="8" t="n">
         <v>65</v>
       </c>
@@ -4259,7 +4260,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="8" t="n">
         <v>66</v>
       </c>
@@ -4282,7 +4283,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="n">
         <v>67</v>
       </c>
@@ -4305,7 +4306,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="8" t="n">
         <v>68</v>
       </c>
@@ -4328,7 +4329,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="8" t="n">
         <v>69</v>
       </c>
@@ -4354,7 +4355,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="8" t="n">
         <v>70</v>
       </c>
@@ -4377,7 +4378,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="8" t="n">
         <v>71</v>
       </c>
@@ -4400,7 +4401,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="8" t="n">
         <v>72</v>
       </c>
@@ -4423,7 +4424,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="n">
         <v>73</v>
       </c>
@@ -4446,7 +4447,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="8" t="n">
         <v>74</v>
       </c>
@@ -4469,7 +4470,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="8" t="n">
         <v>75</v>
       </c>
@@ -4492,7 +4493,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="8" t="n">
         <v>76</v>
       </c>
@@ -4515,7 +4516,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="n">
         <v>77</v>
       </c>
@@ -4541,7 +4542,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="8" t="n">
         <v>78</v>
       </c>
@@ -4567,7 +4568,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="8" t="n">
         <v>79</v>
       </c>
@@ -4590,7 +4591,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="8" t="n">
         <v>80</v>
       </c>
@@ -4613,7 +4614,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="8" t="n">
         <v>81</v>
       </c>
@@ -4636,7 +4637,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="8" t="n">
         <v>82</v>
       </c>
@@ -4659,7 +4660,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="8" t="n">
         <v>83</v>
       </c>
@@ -4682,7 +4683,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="8" t="n">
         <v>84</v>
       </c>
@@ -4705,7 +4706,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="8" t="n">
         <v>85</v>
       </c>
@@ -4728,7 +4729,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="8" t="n">
         <v>86</v>
       </c>
@@ -4751,7 +4752,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="8" t="n">
         <v>87</v>
       </c>
@@ -4774,7 +4775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="8" t="n">
         <v>88</v>
       </c>
@@ -4800,7 +4801,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="8" t="n">
         <v>89</v>
       </c>
@@ -4826,7 +4827,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="8" t="n">
         <v>90</v>
       </c>
@@ -4852,7 +4853,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="8" t="n">
         <v>91</v>
       </c>
@@ -4870,7 +4871,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="8" t="n">
         <v>92</v>
       </c>
@@ -4893,7 +4894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="8" t="n">
         <v>93</v>
       </c>
@@ -4908,7 +4909,7 @@
       <c r="F94" s="13"/>
       <c r="G94" s="13"/>
     </row>
-    <row r="95" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="8" t="n">
         <v>94</v>
       </c>
@@ -4934,7 +4935,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="8" t="n">
         <v>95</v>
       </c>
@@ -4960,7 +4961,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="8" t="n">
         <v>96</v>
       </c>
@@ -4986,7 +4987,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="8" t="n">
         <v>97</v>
       </c>
@@ -5009,7 +5010,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="8" t="n">
         <v>98</v>
       </c>
@@ -5032,7 +5033,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="8" t="n">
         <v>99</v>
       </c>
@@ -5055,7 +5056,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="8" t="n">
         <v>100</v>
       </c>
@@ -5078,7 +5079,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="8" t="n">
         <v>101</v>
       </c>
@@ -5104,7 +5105,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="8" t="n">
         <v>102</v>
       </c>
@@ -5127,7 +5128,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="8" t="n">
         <v>103</v>
       </c>
@@ -5150,7 +5151,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="8" t="n">
         <v>104</v>
       </c>
@@ -5173,7 +5174,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="8" t="n">
         <v>105</v>
       </c>
@@ -5196,7 +5197,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="8" t="n">
         <v>106</v>
       </c>
@@ -5211,7 +5212,7 @@
       <c r="F107" s="13"/>
       <c r="G107" s="13"/>
     </row>
-    <row r="108" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="8" t="n">
         <v>107</v>
       </c>
@@ -5237,7 +5238,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="8" t="n">
         <v>108</v>
       </c>
@@ -5260,7 +5261,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="8" t="n">
         <v>109</v>
       </c>
@@ -5283,7 +5284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="8" t="n">
         <v>110</v>
       </c>
@@ -5303,7 +5304,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="8" t="n">
         <v>111</v>
       </c>
@@ -5326,7 +5327,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="8" t="n">
         <v>112</v>
       </c>
@@ -5349,7 +5350,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="8" t="n">
         <v>113</v>
       </c>
@@ -5372,7 +5373,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="8" t="n">
         <v>114</v>
       </c>
@@ -5395,7 +5396,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="8" t="n">
         <v>115</v>
       </c>
@@ -5418,7 +5419,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="8" t="n">
         <v>116</v>
       </c>
@@ -5441,7 +5442,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="8" t="n">
         <v>117</v>
       </c>
@@ -5464,7 +5465,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="8" t="n">
         <v>118</v>
       </c>
@@ -5487,7 +5488,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="8" t="n">
         <v>119</v>
       </c>
@@ -5502,7 +5503,7 @@
       <c r="F120" s="13"/>
       <c r="G120" s="13"/>
     </row>
-    <row r="121" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="8" t="n">
         <v>120</v>
       </c>
@@ -5528,7 +5529,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="8" t="n">
         <v>121</v>
       </c>
@@ -5551,7 +5552,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="8" t="n">
         <v>122</v>
       </c>
@@ -5574,7 +5575,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="8" t="n">
         <v>123</v>
       </c>
@@ -5597,7 +5598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="8" t="n">
         <v>124</v>
       </c>
@@ -5620,7 +5621,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="8" t="n">
         <v>125</v>
       </c>
@@ -5643,7 +5644,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="8" t="n">
         <v>126</v>
       </c>
@@ -5666,7 +5667,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="8" t="n">
         <v>127</v>
       </c>
@@ -5689,7 +5690,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="8" t="n">
         <v>128</v>
       </c>
@@ -5713,7 +5714,7 @@
       </c>
       <c r="H129" s="19"/>
     </row>
-    <row r="130" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="8" t="n">
         <v>129</v>
       </c>
@@ -5736,7 +5737,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="8" t="n">
         <v>130</v>
       </c>
@@ -5759,7 +5760,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="8" t="n">
         <v>131</v>
       </c>
@@ -5782,7 +5783,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="8" t="n">
         <v>132</v>
       </c>
@@ -5805,7 +5806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="8" t="n">
         <v>133</v>
       </c>
@@ -5828,7 +5829,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="8" t="n">
         <v>134</v>
       </c>
@@ -6644,7 +6645,7 @@
       <c r="B15" s="23" t="s">
         <v>263</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="30" t="n">
         <v>0.54</v>
       </c>
       <c r="D15" s="23" t="s">
@@ -6658,7 +6659,7 @@
       <c r="B16" s="23" t="s">
         <v>266</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="30" t="n">
         <v>1.3628</v>
       </c>
       <c r="D16" s="23" t="s">
@@ -6672,8 +6673,9 @@
       <c r="B17" s="23" t="s">
         <v>269</v>
       </c>
-      <c r="C17" s="23" t="n">
-        <v>-1.344</v>
+      <c r="C17" s="30" t="n">
+        <f aca="false">10^(-1.344/10)</f>
+        <v>0.733837667333538</v>
       </c>
       <c r="D17" s="23" t="s">
         <v>270</v>
@@ -6686,11 +6688,12 @@
       <c r="B18" s="23" t="s">
         <v>272</v>
       </c>
-      <c r="C18" s="23" t="n">
-        <v>-1.7521</v>
+      <c r="C18" s="30" t="n">
+        <f aca="false">10^(-1.7521/20)</f>
+        <v>0.817325408117399</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6700,8 +6703,9 @@
       <c r="B19" s="23" t="s">
         <v>274</v>
       </c>
-      <c r="C19" s="23" t="n">
-        <v>-3.0965</v>
+      <c r="C19" s="30" t="n">
+        <f aca="false">10^(-3.0965/10)</f>
+        <v>0.490173693555492</v>
       </c>
       <c r="D19" s="23" t="s">
         <v>270</v>
@@ -6714,8 +6718,9 @@
       <c r="B20" s="23" t="s">
         <v>276</v>
       </c>
-      <c r="C20" s="23" t="n">
-        <v>-7.1042</v>
+      <c r="C20" s="30" t="n">
+        <f aca="false">10^(-7.1042/20)</f>
+        <v>0.441356980726392</v>
       </c>
       <c r="D20" s="23" t="s">
         <v>270</v>

</xml_diff>